<commit_message>
updated : API Authentication
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -4,7 +4,7 @@
   <x:fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <x:workbookPr codeName="ThisWorkbook"/>
   <x:bookViews>
-    <x:workbookView windowWidth="23040" windowHeight="9000" firstSheet="0" activeTab="2"/>
+    <x:workbookView windowWidth="28800" windowHeight="12180" firstSheet="0" activeTab="1"/>
   </x:bookViews>
   <x:sheets>
     <x:sheet name="Roles" sheetId="1" r:id="rId1"/>
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-08-08T10:26:03.2318906Z</x:t>
+    <x:t>2026-09-28T14:06:13.6523250Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-08-08T10:25:52.2925007Z</x:t>
+    <x:t>2026-09-28T08:28:56.0385018Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-08-08T10:26:04.8705957Z</x:t>
+    <x:t>2026-09-28T14:13:01.2982484Z</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -807,8 +807,8 @@
     <x:cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </x:cellStyles>
   <x:tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1 1" defaultPivotStyle="PivotStylePreset2_Accent1 1">
-    <x:tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="0" xr9:uid="{D912C4B3-9C32-4402-94F0-D5C7ECBC8C95}"/>
-    <x:tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="0" xr9:uid="{963F0849-76DD-41AF-9355-CB1212D29E49}"/>
+    <x:tableStyle name="TableStylePreset3_Accent1 1" pivot="0" count="0" xr9:uid="{8D9C8483-5A64-4691-A339-07560C8A25A5}"/>
+    <x:tableStyle name="PivotStylePreset2_Accent1 1" table="0" count="0" xr9:uid="{FD70FDF4-DA72-4C38-819E-2EF78B968594}"/>
   </x:tableStyles>
   <x:extLst>
     <x:ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -1106,14 +1106,14 @@
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
   <x:dimension ref="A1:F5"/>
-  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="14.4"/>
+  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16.444444" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10.555556" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="16.447619" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="10.552381" style="0" customWidth="1"/>
     <x:col min="3" max="3" width="39" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="54.222222" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="54.219048" style="0" customWidth="1"/>
     <x:col min="5" max="5" width="40.666667" style="0" customWidth="1"/>
-    <x:col min="6" max="6" width="16.111111" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="16.114286" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:6">
@@ -1231,9 +1231,11 @@
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
   <x:dimension ref="A1:D5"/>
-  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="14.4"/>
+  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="12.222222" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.714286" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="11" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="46" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4">
@@ -1321,12 +1323,12 @@
     <x:outlinePr summaryBelow="1" summaryRight="1"/>
   </x:sheetPr>
   <x:dimension ref="A1:D4"/>
-  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="14.4"/>
+  <x:sheetFormatPr defaultColWidth="8.996339" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="16" style="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16.444444" style="0" customWidth="1"/>
-    <x:col min="3" max="3" width="14.888889" style="0" customWidth="1"/>
-    <x:col min="4" max="4" width="8.111111" style="0" customWidth="1"/>
+    <x:col min="1" max="1" width="17.571429" style="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17.714286" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14.885714" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="8.114286" style="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" spans="1:4">

</xml_diff>

<commit_message>
fixed: Report templete and status info
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T14:06:13.6523250Z</x:t>
+    <x:t>2026-09-28T20:53:15.3668258Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T08:28:56.0385018Z</x:t>
+    <x:t>2026-09-28T19:10:09.8993942Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T14:13:01.2982484Z</x:t>
+    <x:t>2026-09-28T20:53:36.6418699Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
added : Patient Authentication, IDOR, Input Validation
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -98,13 +98,13 @@
     <x:t>eyJhbGciOiJSUzI1NiIsImtpZCI6Ilg1ZVhrNHh5...</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T20:53:15.3668258Z</x:t>
+    <x:t>2026-09-29T05:45:17.9386926Z</x:t>
   </x:si>
   <x:si>
     <x:t>2026-07-03T19:49:23.6888430Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T19:10:09.8993942Z</x:t>
+    <x:t>2026-09-29T05:44:27.3617829Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -125,7 +125,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-09-28T20:53:36.6418699Z</x:t>
+    <x:t>2026-09-29T12:25:24.7724424Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>

<commit_message>
added search api end point and its validation
</commit_message>
<xml_diff>
--- a/TestData/UploadFiles/LoginRequest.xlsx
+++ b/TestData/UploadFiles/LoginRequest.xlsx
@@ -116,7 +116,7 @@
     <x:t>2026-09-29T05:44:27.3617829Z</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-07T12:46:16.7198531Z</x:t>
+    <x:t>2026-10-09T13:07:59.8390589Z</x:t>
   </x:si>
   <x:si>
     <x:t>ParentRole</x:t>
@@ -137,7 +137,7 @@
     <x:t>Yes</x:t>
   </x:si>
   <x:si>
-    <x:t>2026-10-08T11:23:03.7539341Z</x:t>
+    <x:t>2026-10-09T13:52:55.2630490Z</x:t>
   </x:si>
 </x:sst>
 </file>

</xml_diff>